<commit_message>
docs: translate check inventory and implementation plan to English
All Chinese content (test names, descriptions, dimensions, categories)
translated to English across both spreadsheets.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/MVA_Check_Inventory.xlsx
+++ b/output/MVA_Check_Inventory.xlsx
@@ -639,17 +639,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>测试</t>
+          <t>Test</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>维度</t>
+          <t>Dimension</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>逻辑</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -691,17 +691,17 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>缺失值分析</t>
+          <t>Missing Value Analysis</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>按变量 × obs_month 计算缺失率，超过阈值（默认 5%）的变量逐月报警，生成 heatmap。缺失率突变可能表示数据提取问题或上游 ETL 变更</t>
+          <t>Missing rate by variable x obs_month, flags variables exceeding threshold (default 5%). Generates heatmap. Sudden changes in missing rate may indicate ETL or data extraction issues</t>
         </is>
       </c>
       <c r="F2" s="6" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>负值 / 下限违规检测</t>
+          <t>Negative / Below-Minimum Detection</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>对 variables.yaml 中有 min 约束的变量（如 balance min=0, dpd min=0）检测低于下限的记录数和占比</t>
+          <t>Detects records below minimum constraints defined in variables.yaml (e.g. balance min=0, dpd min=0). Reports count and percentage of violations</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -771,17 +771,17 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>记录数突变</t>
+          <t>Record Count Spike</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>相邻 obs_month 的记录数变化率超阈值（默认 10%）— 可能表示数据截断、提取不完整或窗口变更</t>
+          <t>Flags obs_months where record count changes by more than threshold (default 10%) vs prior month. May indicate data truncation, incomplete extraction, or window changes</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
@@ -811,17 +811,17 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>异常值检测</t>
+          <t>Outlier Detection</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>对数值型变量使用 IQR（默认 3 倍）或 Z-score 方法检测极端值，排除 Status/Derived/ID 类型和有 valid_values 的变量</t>
+          <t>Detects extreme values in numeric variables using IQR (default 3x) or Z-score method. Excludes Status/Derived/ID types and variables with valid_values</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -851,17 +851,17 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>数据类型检查</t>
+          <t>Data Type Check</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>实际 dtype 与 variables.yaml 预期对比，Date 类型应为 datetime64, Value/Term/Rate 应为 numeric。类型不匹配会导致下游计算错误</t>
+          <t>Compares actual dtype against expected dtype in variables.yaml. Date types should be datetime64, Value/Term/Rate should be numeric. Type mismatches cause downstream calculation errors</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
@@ -891,17 +891,17 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>DPD 缺失率趋势</t>
+          <t>DPD Missing Rate Trend</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>dpd 缺失率按 obs_month 趋势，标记缺失率突变的月份。DPD 缺失影响默认定义（dpd&gt;=90 规则），缺失的记录无法正确识别违约</t>
+          <t>DPD missing rate trend by obs_month, flags months with sudden changes. Missing DPD affects default definition (dpd&gt;=90 rule) - missing records cannot be correctly classified</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -931,17 +931,17 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>DPD 缺失 vs Chargeoff</t>
+          <t>DPD Missing vs Chargeoff</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>dpd=NaN 但 ind_CO=1 的记录，这些账户的违约状态完全依赖 chargeoff indicator，如果 DPD 本应有值则说明数据不完整</t>
+          <t>Records where dpd=NaN but ind_CO=1. Default status relies entirely on chargeoff indicator; if DPD should have a value, this indicates incomplete data</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -971,17 +971,17 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>ind_dft 推导验证</t>
+          <t>ind_dft Derivation Validation</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>重算 ind_dft = (dpd&gt;=90 | cpd&gt;=4 | ind_CO=1) 与实际值对比。Type 1: 应该违约但未标记; Type 2: 标记违约但条件不满足。差异率 &gt; 0 说明定义不一致</t>
+          <t>Recalculates ind_dft = (dpd&gt;=90 | cpd&gt;=4 | ind_CO=1) and compares with actual. Type 1: should be default but not flagged. Type 2: flagged but conditions not met. Discrepancy indicates definition inconsistency</t>
         </is>
       </c>
       <c r="F9" s="8" t="inlineStr">
@@ -1011,17 +1011,17 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>new_to_dft 推导验证</t>
+          <t>new_to_dft Derivation Validation</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>重算 new_to_dft = (ind_dft=1 AND lag_ind_dft=0) 与实际值对比，差异说明 new_to_dft 的推导逻辑与 ind_dft/lag_ind_dft 不一致</t>
+          <t>Recalculates new_to_dft = (ind_dft=1 AND lag_ind_dft=0) and compares with actual. Discrepancy indicates derivation logic inconsistent with ind_dft/lag_ind_dft</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -1051,17 +1051,17 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>连续违约无 Cure</t>
+          <t>Consecutive Default Without Cure</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>同一账户出现多次 new_to_dft=1 且中间 ind_dft 未回到 0，可能是 DPD 在 90 天阈值附近波动导致的虚假 cure/re-default</t>
+          <t>Same account has multiple new_to_dft=1 without ind_dft returning to 0 in between. Likely caused by DPD fluctuating around the 90-day threshold, creating false cure/re-default</t>
         </is>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -1091,17 +1091,17 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>违约率趋势</t>
+          <t>Default Rate Trend</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>ind_dft 率按 obs_month（分母: perf_lvl1∈{0,1} 即 open accounts）; new_to_dft 率按 obs_month（分母: perf_lvl1=0 即 good accounts）。趋势突变可能反映经济周期或定义变更</t>
+          <t>ind_dft rate by obs_month (denominator: perf_lvl1 in {0,1} i.e. open accounts); new_to_dft rate by obs_month (denominator: perf_lvl1=0 i.e. good accounts). Trend breaks may reflect economic cycles or definition changes</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -1131,17 +1131,17 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>DPD 分布趋势</t>
+          <t>DPD Distribution Trend</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>dpd 的 mean / median / 90th percentile 按 obs_month，监控逾期分布是否随时间恶化或改善</t>
+          <t>DPD mean / median / 90th percentile by obs_month. Monitors whether delinquency distribution is worsening or improving over time</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -1171,17 +1171,17 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>CPD vs DPD 一致性</t>
+          <t>CPD vs DPD Consistency</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>cpd 应近似 ceil(dpd/30)，差异说明 cpd 和 dpd 可能是独立推导的，或使用了不同的 cycle 定义（如 billing cycle vs calendar）</t>
+          <t>CPD should approximate ceil(dpd/30). Discrepancy suggests CPD and DPD may be independently derived or use different cycle definitions (billing cycle vs calendar)</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -1211,17 +1211,17 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>ind_closed Cummax 验证</t>
+          <t>ind_closed Cummax Validation</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>关户指标应满足 cummax 逻辑：一旦 ind_closed=1 就不应回到 0。 1→0 的回退说明数据中存在“重开”现象，影响 ERL 终端事件定义</t>
+          <t>Closed indicator should follow cummax logic: once ind_closed=1 it should never revert to 0. Reversals (1-&gt;0) indicate 're-opening' in the data, affecting ERL terminal event definition</t>
         </is>
       </c>
       <c r="F15" s="8" t="inlineStr">
@@ -1251,17 +1251,17 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>ind_CO Cummax 验证</t>
+          <t>ind_CO Cummax Validation</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Chargeoff 指标应满足 cummax 逻辑：一旦 ind_CO=1 就不应回到 0。回退说明 chargeoff 被错误逆转，影响 LGD 计算</t>
+          <t>Chargeoff indicator should follow cummax logic: once ind_CO=1 it should never revert to 0. Reversals indicate incorrectly reversed chargeoffs, affecting LGD calculation</t>
         </is>
       </c>
       <c r="F16" s="8" t="inlineStr">
@@ -1291,17 +1291,17 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>关户但 Balance &gt; 0</t>
+          <t>Closed but Balance &gt; 0</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>ind_closed=1 但 balance &gt; 0，关户后余额应为 0，有余额说明可能是提前关户标记或余额未清零</t>
+          <t>ind_closed=1 but balance &gt; 0. Balance should be zero after closure. Positive balance suggests premature closure flag or balance not zeroed out</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1331,17 +1331,17 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>关户后 Chargeoff</t>
+          <t>Chargeoff After Closure</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>ind_closed=1 后出现 ind_CO=1，chargeoff 通常应在关户之前或同时发生，关户后再 chargeoff 说明时序不一致</t>
+          <t>ind_CO=1 appears after ind_closed=1. Chargeoff should typically occur before or concurrent with closure. Post-closure chargeoff indicates timing inconsistency</t>
         </is>
       </c>
       <c r="F18" s="8" t="inlineStr">
@@ -1371,17 +1371,17 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Chargeoff 但未关户</t>
+          <t>Chargeoff Without Closure</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>ind_CO=1 但 ind_closed=0，chargeoff 通常伴随关户，如果未标记关户则 ERL 终端事件定义可能遗漏这些账户</t>
+          <t>ind_CO=1 but ind_closed=0. Chargeoff typically accompanies closure. If not flagged as closed, ERL terminal event definition may miss these accounts</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1411,17 +1411,17 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>开户日前的 Chargeoff</t>
+          <t>Chargeoff Before Open Date</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>obs_month &lt; dt_opened 的记录中出现 ind_CO=1，账户尚未开户就有 chargeoff 记录，说明日期或数据关联有误</t>
+          <t>Records where obs_month &lt; dt_opened have ind_CO=1. Account not yet opened but has chargeoff record, indicating date or data linkage error</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
@@ -1451,17 +1451,17 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>ind_closed 趋势图</t>
+          <t>ind_closed Trend</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>ind_closed=0 / ind_closed=1 / 总记录数按 obs_month 趋势，监控关户率是否稳定</t>
+          <t>ind_closed=0 / ind_closed=1 / total records by obs_month trend. Monitors whether closure rate is stable</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1491,17 +1491,17 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>ind_CO 趋势图</t>
+          <t>ind_CO Trend</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>ind_CO=0 / ind_CO=1 / 总记录数按 obs_month 趋势，监控 chargeoff 率是否稳定</t>
+          <t>ind_CO=0 / ind_CO=1 / total records by obs_month trend. Monitors whether chargeoff rate is stable</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1531,17 +1531,17 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Balance 负值</t>
+          <t>Negative Balance</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>balance &lt; 0，对于有 min=0 约束的产品（如 mortgage, auto loan），负余额不应存在。可能是 overpayment 或数据错误</t>
+          <t>balance &lt; 0. For products with min=0 constraint (e.g. mortgage, auto loan), negative balance should not exist. May be overpayment or data error</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1571,17 +1571,17 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Balance=0 但 DPD&gt;0</t>
+          <t>Zero Balance with DPD &gt; 0</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>balance=0 但 dpd&gt;0，余额为 0 不应有逾期天数，可能是余额清零后 DPD 未重置，影响违约识别</t>
+          <t>balance=0 but dpd&gt;0. Zero balance should not have delinquency days. DPD may not have been reset after balance cleared, affecting default identification</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1611,17 +1611,17 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>违约时 Balance 缺失</t>
+          <t>Missing Balance at Default</t>
         </is>
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>ind_dft=1 但 balance=NaN，违约账户的余额是 LGD 分母，缺失会导致这些违约被排除在 LGD 估计之外</t>
+          <t>ind_dft=1 but balance=NaN. Defaulted account balance is the LGD denominator. Missing values exclude these defaults from LGD estimation</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1651,17 +1651,17 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Recovery 负值</t>
+          <t>Negative Recovery</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>recovery &lt; 0，负回收通常不应出现，可能是费用或利息被错误计入 recovery 字段</t>
+          <t>recovery &lt; 0. Negative recovery should not normally occur. May be fees or interest incorrectly recorded in the recovery field</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -1696,12 +1696,12 @@
       </c>
       <c r="D27" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>recovery &gt; balance，回收金额超过余额，可能是累计 recovery 跨期计算或数据错误</t>
+          <t>recovery &gt; balance. Recovery amount exceeds balance. May be cumulative cross-period recovery calculation or data error</t>
         </is>
       </c>
       <c r="F27" s="8" t="inlineStr">
@@ -1731,17 +1731,17 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Recovery 趋势</t>
+          <t>Recovery Trend</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>recovery 的 sum / count / mean 按 obs_month，监控回收模式是否稳定，突变可能反映政策或市场变化</t>
+          <t>Recovery sum / count / mean by obs_month. Monitors whether recovery patterns are stable. Sudden changes may reflect policy or market shifts</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -1771,17 +1771,17 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>非违约账户有 Recovery</t>
+          <t>Non-Default with Recovery</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>ind_dft=0 且 ind_CO=0 但 recovery&gt;0，非违约账户不应有回收金额，可能是数据关联错误</t>
+          <t>ind_dft=0 and ind_CO=0 but recovery&gt;0. Non-default accounts should not have recovery amounts. May be a data linkage error</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
@@ -1816,12 +1816,12 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>interest_rate=0 的占比，0% 利率可能是真实值（如促销利率）也可能是缺失值的替代，需要业务确认</t>
+          <t>Percentage of interest_rate=0 records. 0% rate may be genuine (promotional rate) or a missing value substitute. Requires business confirmation</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -1851,17 +1851,17 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>Interest Rate 极端值</t>
+          <t>Extreme Interest Rate</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>interest_rate &gt; 50% 或 &lt; 0，极端利率说明数据可能未转换（如年化 vs 月化）或有录入错误</t>
+          <t>interest_rate &gt; 50% or &lt; 0. Extreme rates suggest data may not be converted (annualized vs monthly) or contains entry errors</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -1891,17 +1891,17 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Balance 趋势</t>
+          <t>Balance Trend</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>balance 的 sum / mean / median 按 obs_month，监控组合余额变化，大幅波动可能反映数据窗口变化或产品组合迁移</t>
+          <t>Balance sum / mean / median by obs_month. Monitors portfolio balance changes. Large fluctuations may reflect data window changes or portfolio composition shifts</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -1931,17 +1931,17 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Interest Rate 趋势</t>
+          <t>Interest Rate Trend</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>interest_rate 的 mean / median / std 按 obs_month。重要：需确认 discounting interest rate 是否与产品 yield rate 一致</t>
+          <t>Interest rate mean / median / std by obs_month. Important: confirm whether discounting interest rate is consistent with product yield rate</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -1971,17 +1971,17 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>next_dft_bal 缺失 / 非违约填充</t>
+          <t>next_dft_bal Missing / Non-Default Fill</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>违约账户(ind_dft=1)的 next_dft_bal 缺失率；非违约账户(ind_dft=0)的 next_dft_bal 应为 NaN。违约余额是 LGD 分子的关键输入，缺失会排除样本</t>
+          <t>Missing rate of next_dft_bal for defaulted accounts (ind_dft=1); non-default accounts (ind_dft=0) should have next_dft_bal=NaN. Default balance is a key LGD numerator input; missing values exclude samples</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -2011,17 +2011,17 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>next_dft_bal 负值</t>
+          <t>Negative next_dft_bal</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>next_dft_bal &lt; 0，违约时的负余额不合理，会导致 LGD 计算失真</t>
+          <t>next_dft_bal &lt; 0. Negative balance at default is illogical and will distort LGD calculation</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -2051,17 +2051,17 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>next_dft_bal vs Balance 一致性</t>
+          <t>next_dft_bal vs Balance Consistency</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>在 new_to_dft=1 时比较 next_dft_bal 与 balance，首次违约时两者应接近（差异 &gt;10% 报警），大差异说明取值时点或推导逻辑不同</t>
+          <t>Compares next_dft_bal vs balance at new_to_dft=1. At first default, both should be close (flags &gt;10% difference). Large gaps indicate different valuation timing or derivation logic</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2091,17 +2091,17 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>next_dft_bal=0 的违约账户</t>
+          <t>Zero next_dft_bal at Default</t>
         </is>
       </c>
       <c r="D37" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>ind_dft=1 但 next_dft_bal=0，违约时余额为 0 使 LGD 无定义，检查是否是数据错误或已全额回收后才标违约</t>
+          <t>ind_dft=1 but next_dft_bal=0. Zero balance at default makes LGD undefined. Check whether this is data error or full recovery before default flag</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -2131,17 +2131,17 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>mths_to_dft 违约账户缺失</t>
+          <t>mths_to_dft Missing at Default</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>ind_dft=1 的记录中 mths_to_dft 缺失率，该变量用于 PD term structure 估计，缺失会减少可用违约样本</t>
+          <t>Missing rate of mths_to_dft for records where ind_dft=1. Used for PD term structure estimation; missing values reduce usable default samples</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -2171,17 +2171,17 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>mths_to_dft 负值</t>
+          <t>Negative mths_to_dft</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>mths_to_dft &lt; 0，逻辑上不可能出现负的“到违约月数”，通常是 dt_next_dft &lt; obs_month 的推导错误</t>
+          <t>mths_to_dft &lt; 0. Logically impossible to have negative months-to-default. Usually a derivation error where dt_next_dft &lt; obs_month</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
@@ -2211,17 +2211,17 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>mths_to_dft 分布趋势</t>
+          <t>mths_to_dft Distribution Trend</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>mths_to_dft 的 mean / median 按 obs_month，监控到违约的平均时长变化，趋势性下降可能反映风险恶化</t>
+          <t>mths_to_dft mean / median by obs_month. Monitors changes in average time-to-default. Declining trend may reflect risk deterioration</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -2251,17 +2251,17 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>mths_to_dft vs MOB 一致性</t>
+          <t>mths_to_dft vs MOB Consistency</t>
         </is>
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>在 new_to_dft=1 时比较 mths_to_dft 与 mob，首次违约时两者应近似（|差| &gt; 2 报警），大差异说明推导使用了不同的参考日期</t>
+          <t>Compares mths_to_dft vs mob at new_to_dft=1. At first default both should be similar (flags |diff| &gt; 2). Large gaps indicate different reference dates in derivation</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -2291,17 +2291,17 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>perf_lvl1 重算验证</t>
+          <t>perf_lvl1 Recalculation Validation</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>按推导优先级重算 perf_lvl1 与实际值对比，差异率 &gt; 0 说明推导逻辑与实际标记不一致</t>
+          <t>Recalculates perf_lvl1 using derivation priority rules and compares with actual. Discrepancy &gt; 0 indicates derivation logic inconsistent with actual flags</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -2331,17 +2331,17 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>perf_lvl1 分布趋势</t>
+          <t>perf_lvl1 Distribution Trend</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>perf_lvl1 各 level（0=Good, 1=Default, 2=Closed, 3=Exclusion）占比按 obs_month，监控组合结构变化</t>
+          <t>perf_lvl1 level distribution (0=Good, 1=Default, 2=Closed, 3=Exclusion) by obs_month. Monitors portfolio composition changes</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -2371,17 +2371,17 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Functional 账户占比</t>
+          <t>Functional Account Proportion</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>perf_lvl1=0 的占比，functional 账户应是主体（&gt;50%），过低说明排除/关户过多，下游模型样本可能不足</t>
+          <t>Percentage of perf_lvl1=0 (functional accounts). Should be majority (&gt;50%). Low ratio indicates excessive exclusions/closures; downstream model samples may be insufficient</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -2411,17 +2411,17 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>perf_lvl1 × perf_lvl2 交叉表</t>
+          <t>perf_lvl1 x perf_lvl2 Cross-Tab</t>
         </is>
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>交叉表验证映射关系。有效组合: (0,0) Good/stays good, (0,1) Good/defaults 12m, (1,1) Default/DPD, (1,2) Default/CO, (2,0) Not open, (2,1) CO, (2,2) Closed</t>
+          <t>Cross-tabulation validates mapping. Valid combinations: (0,0) Good/stays good, (0,1) Good/defaults 12m, (1,1) Default/DPD, (1,2) Default/CO, (2,0) Not open, (2,1) CO, (2,2) Closed</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -2451,17 +2451,17 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Score-Default 单调性</t>
+          <t>Score-Default Monotonicity</t>
         </is>
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>按 score 分段计算 IFRS 9 default rate，score 越高 default rate 应越低（单调性）。如果单调性破坏，说明 score 对 IFRS 9 default 没有区分力</t>
+          <t>Calculates IFRS 9 default rate by score segment. Higher score should have lower default rate (monotonicity). Broken monotonicity indicates score lacks discriminatory power for IFRS 9 default</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -2491,17 +2491,17 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>高分段违约率异常</t>
+          <t>High-Score Segment Default Rate</t>
         </is>
       </c>
       <c r="D47" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>最低风险分段的 default rate &gt; 阈值（默认 2%），如果最“安全”的分段违约率仍然很高，说明 score 整体区分力不足</t>
+          <t>Lowest risk segment default rate &gt; threshold (default 2%). If the 'safest' segment has high default rate, overall score discriminatory power is insufficient</t>
         </is>
       </c>
       <c r="F47" s="8" t="inlineStr">
@@ -2531,17 +2531,17 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Score 分段 Default Rate 稳定性</t>
+          <t>Score Segment Default Rate Stability</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>按 score 分段 + obs_month 计算 default rate 趋势，如果某些分段的 default rate 大幅波动，可能是 definition misalignment 导致</t>
+          <t>Default rate by score segment x obs_month. If certain segments show large fluctuations, may indicate definition misalignment</t>
         </is>
       </c>
       <c r="F48" s="8" t="inlineStr">
@@ -2571,17 +2571,17 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>Score 极端值</t>
+          <t>Score Extreme Values</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>score=0 或 score&gt;1000 的记录数，极端值应从最终 score 计算中排除，可能是缺失值替代或系统错误</t>
+          <t>Records with score=0 or score&gt;1000. Extreme values should be excluded from final score calculation. May be missing value substitutes or system errors</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
@@ -2611,17 +2611,17 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>score_orig 缺失率趋势</t>
+          <t>score_orig Missing Rate Trend</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
-          <t>score_orig 缺失率按 obs_month，缺失率突变可能表示评分模型更新、评分卡切换或上游数据源变更</t>
+          <t>score_orig missing rate by obs_month. Sudden changes may indicate scoring model update, scorecard switch, or upstream data source change</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
@@ -2651,17 +2651,17 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>score_bhv 缺失率趋势</t>
+          <t>score_bhv Missing Rate Trend</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>score_bhv 缺失率按 obs_month，score 文件 merge 不完整会导致缺失率上升，缺失意味着 alignment 过程有账户没覆盖到</t>
+          <t>score_bhv missing rate by obs_month. Incomplete score file merge causes rising missing rate. Missing means alignment process has uncovered accounts</t>
         </is>
       </c>
       <c r="F51" s="8" t="inlineStr">
@@ -2691,17 +2691,17 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>Score 分布突变检测</t>
+          <t>Score Distribution Drift Detection</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
-          <t>score 的 mean / std 按 obs_month，评分卡更新会导致分布断层（mean 跳变、std 突变），需要在 alignment 中区分新旧评分卡</t>
+          <t>Score mean / std by obs_month. Scorecard updates cause distribution breaks (mean jumps, std spikes). Need to distinguish old vs new scorecards in alignment</t>
         </is>
       </c>
       <c r="F52" s="8" t="inlineStr">
@@ -2731,17 +2731,17 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>dt_opened 缺失率</t>
+          <t>dt_opened Missing Rate</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>dt_opened 缺失率按 obs_month，缺失的开户日导致 perf_lvl1 被排除、mob 无法计算、Loan Term 缺失</t>
+          <t>dt_opened missing rate by obs_month. Missing open date causes perf_lvl1 exclusion, mob cannot be calculated, loan term is missing</t>
         </is>
       </c>
       <c r="F53" s="8" t="inlineStr">
@@ -2776,12 +2776,12 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>开户日期晚于观察月，账户尚未开户就出现在数据中，导致 mob 为负值，通常是 imputation 或数据关联错误</t>
+          <t>Open date later than observation month. Account not yet opened appearing in data causes negative mob. Usually imputation or data linkage error</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -2811,17 +2811,17 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>MOB 负值</t>
+          <t>Negative MOB</t>
         </is>
       </c>
       <c r="D55" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>mob = obs_month - dt_opened &lt; 0，DO2 的下游结果，负 mob 会影响 DF cohort 和 SICR stage allocation</t>
+          <t>mob = obs_month - dt_opened &lt; 0. Downstream result of DO2. Negative mob affects DF cohort and SICR stage allocation</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
@@ -2856,12 +2856,12 @@
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>balance &gt; 120% × ln_value 的记录，balance 显著超过贷款价值可能是资本化利息/费用或数据错误，对 EAD 估计有直接影响</t>
+          <t>balance &gt; 120% x ln_value records. Balance significantly exceeding loan value may be capitalized interest/fees or data error. Direct impact on EAD estimation</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
@@ -2891,17 +2891,17 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>Loan Value 恒定性</t>
+          <t>Loan Value Consistency Over Time</t>
         </is>
       </c>
       <c r="D57" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>同一账户 ln_value 在不同 obs_month 是否变化，贷款价值在发放时确定，变化说明可能有 restructure、top-up 或数据 join 问题</t>
+          <t>Whether ln_value changes across obs_months for the same account. Loan value is fixed at origination; changes indicate restructure, top-up, or data join issues</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
@@ -2931,17 +2931,17 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>Loan Value 趋势</t>
+          <t>Loan Value Trend</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>ln_value 的 mean / median 按 obs_month，监控新发放贷款的平均金额变化，大幅变化可能反映产品策略或市场变化</t>
+          <t>ln_value mean / median by obs_month. Monitors average new origination amount changes. Large shifts may reflect product strategy or market changes</t>
         </is>
       </c>
       <c r="F58" s="9" t="inlineStr">
@@ -2971,17 +2971,17 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>Booked Amount 恒定性</t>
+          <t>Booked Amount Consistency Over Time</t>
         </is>
       </c>
       <c r="D59" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>同一账户 booked_amt 在不同 obs_month 是否变化，booked_amt 是发放时固定金额，变化说明数据 join 或 restructure 问题</t>
+          <t>Whether booked_amt changes across obs_months for the same account. Booked amount is fixed at origination; changes indicate data join or restructure issues</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
@@ -3016,12 +3016,12 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>booked_amt 与 ln_value 差异 &gt;10%，对于非循环产品两者应接近，大差异说明字段定义不同或有数据问题</t>
+          <t>booked_amt vs ln_value difference &gt;10%. For non-revolving products both should be close. Large gap indicates different field definitions or data issues</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
@@ -3051,17 +3051,17 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>Restructure Rate 趋势</t>
+          <t>Restructure Rate Trend</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>ind_restructure=1 的占比按 obs_month，突增可能反映经济事件（如 COVID）或政策调整。restructure 账户需要在 Score Alignment 中特殊处理</t>
+          <t>ind_restructure=1 rate by obs_month. Sudden increase may reflect economic events (e.g. COVID) or policy changes. Restructured accounts need special treatment in Score Alignment</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
@@ -3091,17 +3091,17 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>未标记的 Restructure</t>
+          <t>Unmarked Restructure</t>
         </is>
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>ln_term 发生变化但 ind_restructure 始终为 0，term 变更通常伴随 restructure，未标记说明 restructure flag 可能不完整</t>
+          <t>ln_term changes but ind_restructure remains 0. Term changes typically accompany restructure; unmarked cases indicate restructure flag may be incomplete</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -3136,12 +3136,12 @@
       </c>
       <c r="D63" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>无故消失的账户（最后记录 &lt; 全局最大 obs_month，且非 closed/CO/default），这些账户的 outcome 未知，影响 ERL 和 DF 的 survival analysis</t>
+          <t>Accounts that disappear without explanation (last record &lt; global max obs_month, not closed/CO/default). Outcome is unknown, affecting ERL and DF estimation</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -3171,17 +3171,17 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>消失账户趋势</t>
+          <t>Disappeared Account Trend</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>每月新消失账户数和占比，消失账户集中在特定月份可能说明该月数据提取不完整或有系统性问题</t>
+          <t>Monthly count and percentage of newly disappeared accounts. Concentration in specific months may indicate incomplete data extraction or systematic issues</t>
         </is>
       </c>
       <c r="F64" s="6" t="inlineStr">
@@ -3211,17 +3211,17 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>单条记录账户</t>
+          <t>Single-Record Accounts</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>只有一条记录的 acct_id，单条记录无法构建 survival 曲线，对 ERL 和 PD 估计无贡献但占用 population</t>
+          <t>Accounts with only one record. Single records cannot build survival curves; contribute nothing to ERL and PD estimation but occupy population</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -3251,17 +3251,17 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>记录间断检测</t>
+          <t>Record Gap Detection</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>同一账户的 obs_month 序列中出现跳月（gap &gt; 1 month），缺失月份会导致 transition matrix 中断，影响 PD/ERL</t>
+          <t>Gaps in obs_month sequence for same account (gap &gt; 1 month). Missing months interrupt transition matrices, affecting PD/ERL estimation</t>
         </is>
       </c>
       <c r="F66" s="8" t="inlineStr">
@@ -3291,17 +3291,17 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>不完整观察月</t>
+          <t>Incomplete Observation Month</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>某月的账户数低于中位数的 50%，该月数据可能不完整，应考虑从分析中排除</t>
+          <t>Month with account count below 50% of median. Data for that month may be incomplete; consider excluding from analysis</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -3331,17 +3331,17 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>消失账户画像</t>
+          <t>Disappeared Account Profile</t>
         </is>
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>按最终状态分类消失账户（default / closed / exclusion / censored），了解消失原因的分布，censored 占比过高需要关注</t>
+          <t>Classifies disappeared accounts by final status (default / closed / exclusion / censored). High censored proportion warrants attention</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
@@ -3376,12 +3376,12 @@
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>dt_opened 早于数据窗口起点的账户，这些账户的早期历史缺失，mob 的早期阶段 transition 不可观察</t>
+          <t>Accounts with dt_opened earlier than data window start. Early history is missing; early-stage mob transitions are unobservable</t>
         </is>
       </c>
       <c r="F69" s="6" t="inlineStr">
@@ -3411,17 +3411,17 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>违约后追踪期</t>
+          <t>Post-Default Tracking Period</t>
         </is>
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>ind_dft=1 后的后续观察记录数是否 &gt;= 12 个月，LGD 估计需要足够的 recovery 追踪期，追踪不足会低估 recovery</t>
+          <t>Whether records post ind_dft=1 have &gt;= 12 months of follow-up. LGD estimation requires sufficient recovery tracking period; insufficient tracking underestimates recovery</t>
         </is>
       </c>
       <c r="F70" s="8" t="inlineStr">
@@ -3451,17 +3451,17 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>时序异常检测</t>
+          <t>Time Series Anomaly Detection</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>对指定变量（ind_closed, ind_CO, recovery, balance, dpd）的月度聚合值进行 Z-score 异常检测，超过阈值（默认 2.5σ）的月份标记为异常</t>
+          <t>Z-score anomaly detection on monthly aggregates of specified variables (ind_closed, ind_CO, recovery, balance, dpd). Flags values exceeding threshold (default 2.5)</t>
         </is>
       </c>
       <c r="F71" s="6" t="inlineStr">
@@ -3491,17 +3491,17 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>maturity_dt 缺失率</t>
+          <t>maturity_dt Missing Rate</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>maturity_dt 缺失率，term 产品必须有到期日，缺失影响 DF cohort 分组和 ERL 终端事件计算</t>
+          <t>maturity_dt missing rate. Term products must have maturity date; missing affects DF cohort grouping and ERL terminal event calculation</t>
         </is>
       </c>
       <c r="F72" s="8" t="inlineStr">
@@ -3536,12 +3536,12 @@
       </c>
       <c r="D73" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>到期日早于开户日，逻辑上不可能，说明日期字段有录入或转换错误</t>
+          <t>Maturity date earlier than open date. Logically impossible; indicates date field entry or conversion error</t>
         </is>
       </c>
       <c r="F73" s="8" t="inlineStr">
@@ -3571,17 +3571,17 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>到期但仍 Open</t>
+          <t>Past Maturity but Still Open</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
-          <t>maturity_dt &lt; obs_month 且 ind_closed=0 且 perf_lvl1=0，已过到期日但账户仍为 functional/open，影响 ERL 终端事件定义</t>
+          <t>maturity_dt &lt; obs_month and ind_closed=0 and perf_lvl1=0. Past maturity but account still functional/open, suggests maturity not enforced or date error</t>
         </is>
       </c>
       <c r="F74" s="8" t="inlineStr">
@@ -3611,17 +3611,17 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>maturity_dt 时序一致性</t>
+          <t>maturity_dt Temporal Consistency</t>
         </is>
       </c>
       <c r="D75" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E75" s="4" t="inlineStr">
         <is>
-          <t>同一账户 maturity_dt 在不同 obs_month 变化（排除 ind_restructure=1），非 restructure 情况下到期日不应变化</t>
+          <t>maturity_dt changes across obs_months for same account (excluding ind_restructure=1). Without restructure, maturity date should not change</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
@@ -3651,17 +3651,17 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>Loan Term 范围</t>
+          <t>Loan Term Range</t>
         </is>
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
-          <t>ln_term 是否在产品合理范围内（如 MG: 60-360 月, AL: 12-84 月），超范围值说明可能是不同产品混入或录入错误</t>
+          <t>Whether ln_term falls within reasonable product range (e.g. MG: 60-360 months, AL: 12-84 months). Out-of-range values suggest product mix contamination or entry errors</t>
         </is>
       </c>
       <c r="F76" s="6" t="inlineStr">
@@ -3691,17 +3691,17 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>Loan Term 增长</t>
+          <t>Loan Term Growth</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E77" s="4" t="inlineStr">
         <is>
-          <t>同一账户 ln_term 随时间增大但 ind_restructure≠1，term 增长通常伴随 restructure，未标记说明数据不一致</t>
+          <t>ln_term increases over time for same account but ind_restructure!=1. Term growth typically accompanies restructure; unmarked cases indicate data inconsistency</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
@@ -3731,17 +3731,17 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>Remaining Term 负值</t>
+          <t>Negative Remaining Term</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>remaining_term &lt; 0，剩余期限为负说明账户已过到期日，应已关户或有 restructure</t>
+          <t>remaining_term &lt; 0. Negative remaining term indicates account is past maturity; should be closed or restructured</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
@@ -3776,12 +3776,12 @@
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
         <is>
-          <t>mob + remaining_term 与 ln_term 差异 &gt; 2 个月，三者应满足一致性约束，差异说明某个字段推导有误</t>
+          <t>mob + remaining_term vs ln_term difference &gt; 2 months. The three should satisfy consistency constraint; discrepancy indicates derivation error in one field</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
@@ -3816,12 +3816,12 @@
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
-          <t>remaining_term ≈ maturity_dt - obs_month，两种计算方式应一致，差异 &gt; 2 个月报警</t>
+          <t>remaining_term should approximate maturity_dt - obs_month. Two calculation methods should agree; flags difference &gt; 2 months</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
@@ -3851,17 +3851,17 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>Credit Limit 缺失率</t>
+          <t>Credit Limit Missing Rate</t>
         </is>
       </c>
       <c r="D81" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
         <is>
-          <t>credit_limit 缺失率，revolving 产品的额度是 EAD CCF 计算的关键输入，缺失会导致 EAD 无法估计</t>
+          <t>credit_limit missing rate. Credit limit is a key input for EAD CCF calculation in revolving products; missing values prevent EAD estimation</t>
         </is>
       </c>
       <c r="F81" s="8" t="inlineStr">
@@ -3896,12 +3896,12 @@
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
-          <t>credit_limit=0 或 &lt;0，零或负额度不合理，可能是关户后额度清零或数据错误</t>
+          <t>credit_limit=0 or &lt;0. Zero or negative limit is illogical; may be post-closure limit zeroing or data error</t>
         </is>
       </c>
       <c r="F82" s="8" t="inlineStr">
@@ -3931,17 +3931,17 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>Credit Limit 极端值</t>
+          <t>Credit Limit Extreme Values</t>
         </is>
       </c>
       <c r="D83" s="5" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
       <c r="E83" s="4" t="inlineStr">
         <is>
-          <t>异常高的 credit_limit，可能是货币未转换（如 peso vs USD）或系统录入错误</t>
+          <t>Abnormally high credit_limit. May be unconverted currency (e.g. peso vs USD) or system entry error</t>
         </is>
       </c>
       <c r="F83" s="6" t="inlineStr">
@@ -3971,17 +3971,17 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Utilization 分布</t>
+          <t>Utilization Distribution</t>
         </is>
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
-          <t>balance / credit_limit 分布，utilization &gt;1（超额使用）和 ≤0 的占比。CCF 计算依赖 utilization 分布的合理性</t>
+          <t>Distribution of balance / credit_limit. Percentage with utilization &gt;1 (over-limit) and &lt;=0. CCF calculation depends on utilization distribution being reasonable</t>
         </is>
       </c>
       <c r="F84" s="8" t="inlineStr">
@@ -4011,17 +4011,17 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Credit Limit 变动</t>
+          <t>Credit Limit Volatility</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="E85" s="4" t="inlineStr">
         <is>
-          <t>同一账户 credit_limit 的变化频率和幅度，频繁变动可能反映额度管理策略，但也可能是数据问题</t>
+          <t>Frequency and magnitude of credit_limit changes for same account. Frequent changes may reflect limit management strategy but could also indicate data issues</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
@@ -4051,17 +4051,17 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Credit Limit 趋势</t>
+          <t>Credit Limit Trend</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
-          <t>credit_limit 均值按 obs_month，监控组合额度变化趋势</t>
+          <t>credit_limit mean by obs_month. Monitors portfolio limit trend changes</t>
         </is>
       </c>
       <c r="F86" s="9" t="inlineStr">
@@ -4119,7 +4119,7 @@
       </c>
       <c r="B1" s="22" t="inlineStr">
         <is>
-          <t>总数</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="C1" s="22" t="inlineStr">
@@ -4139,17 +4139,17 @@
       </c>
       <c r="F1" s="22" t="inlineStr">
         <is>
-          <t>联动关系</t>
+          <t>Cross-variable</t>
         </is>
       </c>
       <c r="G1" s="22" t="inlineStr">
         <is>
-          <t>趋势</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="H1" s="22" t="inlineStr">
         <is>
-          <t>变量本身</t>
+          <t>Variable-level</t>
         </is>
       </c>
     </row>

</xml_diff>